<commit_message>
regex for undated updated
</commit_message>
<xml_diff>
--- a/testing-column.xlsx
+++ b/testing-column.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\leading-zeros-dates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4239EE-3128-4D94-B46B-0B8EC68C8904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D01763A-87DE-45A7-9ED1-22BF114E0286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25770" yWindow="150" windowWidth="25785" windowHeight="20685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <t>Solved</t>
   </si>
   <si>
-    <t>FullDate</t>
+    <t>Convert Us</t>
   </si>
   <si>
     <t>Expected Result</t>
@@ -37,10 +37,10 @@
     <t>FormattedFullDate1</t>
   </si>
   <si>
-    <t>FormattedFullDate</t>
-  </si>
-  <si>
-    <t>Check Me</t>
+    <t>FormattedFullDate2</t>
+  </si>
+  <si>
+    <t>Check Me1</t>
   </si>
   <si>
     <t>y</t>
@@ -953,13 +953,12 @@
   <dimension ref="A1:G118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.28515625" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+    <col min="6" max="6" width="24.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>